<commit_message>
fix rp5页面Chinese station 逻辑错误，应该只关注20:00Tn和Tx
</commit_message>
<xml_diff>
--- a/气象/蒙古存档.xlsx
+++ b/气象/蒙古存档.xlsx
@@ -26119,49 +26119,88 @@
       <c r="A560" s="1" t="n">
         <v>46319</v>
       </c>
-      <c r="B560" t="n">
+      <c r="B560" s="0" t="n">
         <v>-9.4</v>
       </c>
-      <c r="C560" t="n">
+      <c r="C560" s="0" t="n">
         <v>-8.300000000000001</v>
       </c>
-      <c r="D560" t="n">
+      <c r="D560" s="0" t="n">
         <v>-20.4</v>
       </c>
-      <c r="E560" t="n">
+      <c r="E560" s="0" t="n">
         <v>-15.8</v>
       </c>
-      <c r="F560" t="n">
+      <c r="F560" s="0" t="n">
         <v>-20.6</v>
       </c>
-      <c r="G560" t="n">
+      <c r="G560" s="0" t="n">
         <v>-13.7</v>
       </c>
-      <c r="H560" t="n">
+      <c r="H560" s="0" t="n">
         <v>-12.1</v>
       </c>
-      <c r="I560" t="n">
+      <c r="I560" s="0" t="n">
         <v>-7.4</v>
       </c>
-      <c r="J560" t="n">
+      <c r="J560" s="0" t="n">
         <v>-21</v>
       </c>
-      <c r="K560" t="n">
+      <c r="K560" s="0" t="n">
         <v>-22.2</v>
       </c>
-      <c r="L560" t="n">
+      <c r="L560" s="0" t="n">
         <v>-18.5</v>
       </c>
-      <c r="M560" t="n">
+      <c r="M560" s="0" t="n">
         <v>-12.9</v>
       </c>
-      <c r="N560" t="n">
+      <c r="N560" s="0" t="n">
         <v>-11.1</v>
       </c>
     </row>
     <row r="561">
       <c r="A561" s="1" t="n">
         <v>46320</v>
+      </c>
+      <c r="B561" t="n">
+        <v>-10.9</v>
+      </c>
+      <c r="C561" t="n">
+        <v>-11.8</v>
+      </c>
+      <c r="D561" t="n">
+        <v>-21.1</v>
+      </c>
+      <c r="E561" t="n">
+        <v>-20</v>
+      </c>
+      <c r="F561" t="n">
+        <v>-24</v>
+      </c>
+      <c r="G561" t="n">
+        <v>-15.8</v>
+      </c>
+      <c r="H561" t="n">
+        <v>-10.1</v>
+      </c>
+      <c r="I561" t="n">
+        <v>-9.1</v>
+      </c>
+      <c r="J561" t="n">
+        <v>-20.5</v>
+      </c>
+      <c r="K561" t="n">
+        <v>-24.7</v>
+      </c>
+      <c r="L561" t="n">
+        <v>-19.6</v>
+      </c>
+      <c r="M561" t="n">
+        <v>-16.2</v>
+      </c>
+      <c r="N561" t="n">
+        <v>-10.7</v>
       </c>
     </row>
     <row r="562">
@@ -52586,49 +52625,88 @@
       <c r="A560" s="1" t="n">
         <v>46319</v>
       </c>
-      <c r="B560" t="n">
+      <c r="B560" s="0" t="n">
         <v>4.4</v>
       </c>
-      <c r="C560" t="n">
+      <c r="C560" s="0" t="n">
         <v>0.7</v>
       </c>
-      <c r="D560" t="n">
+      <c r="D560" s="0" t="n">
         <v>-6.5</v>
       </c>
-      <c r="E560" t="n">
+      <c r="E560" s="0" t="n">
         <v>-4.6</v>
       </c>
-      <c r="F560" t="n">
+      <c r="F560" s="0" t="n">
         <v>-8.199999999999999</v>
       </c>
-      <c r="G560" t="n">
+      <c r="G560" s="0" t="n">
         <v>-2.9</v>
       </c>
-      <c r="H560" t="n">
+      <c r="H560" s="0" t="n">
         <v>2.6</v>
       </c>
-      <c r="I560" t="n">
+      <c r="I560" s="0" t="n">
         <v>3.6</v>
       </c>
-      <c r="J560" t="n">
+      <c r="J560" s="0" t="n">
         <v>-7</v>
       </c>
-      <c r="K560" t="n">
+      <c r="K560" s="0" t="n">
         <v>-6.4</v>
       </c>
-      <c r="L560" t="n">
+      <c r="L560" s="0" t="n">
         <v>-3.2</v>
       </c>
-      <c r="M560" t="n">
+      <c r="M560" s="0" t="n">
         <v>-3.8</v>
       </c>
-      <c r="N560" t="n">
+      <c r="N560" s="0" t="n">
         <v>2.2</v>
       </c>
     </row>
     <row r="561">
       <c r="A561" s="1" t="n">
         <v>46320</v>
+      </c>
+      <c r="B561" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="C561" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D561" t="n">
+        <v>-6.6</v>
+      </c>
+      <c r="E561" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="F561" t="n">
+        <v>-10.2</v>
+      </c>
+      <c r="G561" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="H561" t="n">
+        <v>2</v>
+      </c>
+      <c r="I561" t="n">
+        <v>3</v>
+      </c>
+      <c r="J561" t="n">
+        <v>-3</v>
+      </c>
+      <c r="K561" t="n">
+        <v>-7.5</v>
+      </c>
+      <c r="L561" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="M561" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="N561" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="562">
@@ -70251,57 +70329,104 @@
       <c r="A318" s="1" t="n">
         <v>46319</v>
       </c>
-      <c r="B318" t="n">
+      <c r="B318" s="0" t="n">
         <v>-3.79</v>
       </c>
-      <c r="C318" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="D318" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="E318" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="F318" t="n">
+      <c r="C318" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D318" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="E318" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F318" s="0" t="n">
         <v>-13.84</v>
       </c>
-      <c r="G318" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="H318" t="n">
+      <c r="G318" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H318" s="0" t="n">
         <v>-4.9</v>
       </c>
-      <c r="I318" t="n">
+      <c r="I318" s="0" t="n">
         <v>-2.58</v>
       </c>
-      <c r="J318" t="n">
+      <c r="J318" s="0" t="n">
         <v>-14.54</v>
       </c>
-      <c r="K318" t="n">
+      <c r="K318" s="0" t="n">
         <v>-14.74</v>
       </c>
-      <c r="L318" t="n">
+      <c r="L318" s="0" t="n">
         <v>-12.54</v>
       </c>
-      <c r="M318" t="n">
+      <c r="M318" s="0" t="n">
         <v>-9.130000000000001</v>
       </c>
-      <c r="N318" t="n">
+      <c r="N318" s="0" t="n">
         <v>-5.56</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="n">
         <v>46320</v>
+      </c>
+      <c r="B319" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F319" t="n">
+        <v>-17.93</v>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H319" t="n">
+        <v>-4.01</v>
+      </c>
+      <c r="I319" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="J319" t="n">
+        <v>-10.73</v>
+      </c>
+      <c r="K319" t="n">
+        <v>-15.45</v>
+      </c>
+      <c r="L319" t="n">
+        <v>-12.43</v>
+      </c>
+      <c r="M319" t="n">
+        <v>-11.2</v>
+      </c>
+      <c r="N319" t="n">
+        <v>-5.44</v>
       </c>
     </row>
     <row r="320">

</xml_diff>